<commit_message>
nuke CONN_OBSERVER_DISCONN, always splice remove
</commit_message>
<xml_diff>
--- a/Disconnect tests.xlsx
+++ b/Disconnect tests.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_NewDudo\Dudo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC634C0-E194-4E29-945C-F505B081026E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79C49F9-A33F-4837-82A4-268A78BEFB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="29">
   <si>
     <t>Observer</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Bid made: NO</t>
   </si>
   <si>
-    <t>Bid made: YES</t>
-  </si>
-  <si>
     <t>disconnect / reconnect</t>
   </si>
   <si>
@@ -64,6 +61,57 @@
   </si>
   <si>
     <t>Bids, doubt</t>
+  </si>
+  <si>
+    <t>Countdown?</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>splice</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>restore state</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>start a new Round</t>
+  </si>
+  <si>
+    <t>mark Round as Time-out</t>
+  </si>
+  <si>
+    <t>lift his cup</t>
+  </si>
+  <si>
+    <t>change cup image?</t>
+  </si>
+  <si>
+    <t>nextRoundMustSay = false</t>
+  </si>
+  <si>
+    <t>PostRound -&gt; clean up DEFERRED</t>
+  </si>
+  <si>
+    <t>mark TIME_OUT_DEFERRED</t>
+  </si>
+  <si>
+    <t>process doubt as usual</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -79,15 +127,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -95,12 +155,149 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,112 +578,386 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:E27"/>
+  <dimension ref="B2:J32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="3.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.5703125" customWidth="1"/>
     <col min="5" max="5" width="21.7109375" customWidth="1"/>
     <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="12" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="9"/>
+      <c r="C4" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="11"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="3"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+      <c r="E5" s="1"/>
+      <c r="F5" s="4"/>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="3"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="4"/>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="3"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="4"/>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="6"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="E9" s="2"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="15" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C11" t="s">
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="9"/>
+      <c r="C11" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="3"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D13" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="4"/>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="3"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="1"/>
+      <c r="F13" s="4"/>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="3"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D14" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="4"/>
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="9"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="11"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="3"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="3"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="4"/>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="3"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="4"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="9"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E17" t="s">
+      <c r="E20" s="10"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="11"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="3"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="4"/>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="3"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="E18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D19" t="s">
+      <c r="F22" s="4"/>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="3"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="9"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D26" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
+      <c r="E24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="3"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="3"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="6"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CloudSQL to Firestore first cut
</commit_message>
<xml_diff>
--- a/Disconnect tests.xlsx
+++ b/Disconnect tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_NewDudo\Dudo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C79C49F9-A33F-4837-82A4-268A78BEFB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2C2064-CD98-4E56-87D3-CC1723E628A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="30">
   <si>
     <t>Observer</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>OK</t>
+  </si>
+  <si>
+    <t>no, I'll watch -&gt; no cup shown</t>
   </si>
 </sst>
 </file>
@@ -578,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J32"/>
+  <dimension ref="B2:L32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="3.7109375" customWidth="1"/>
@@ -589,7 +592,7 @@
     <col min="8" max="8" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="G2" t="s">
         <v>12</v>
       </c>
@@ -600,7 +603,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
         <v>0</v>
       </c>
@@ -611,7 +614,7 @@
       <c r="G3" s="13"/>
       <c r="H3" s="14"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
         <v>1</v>
@@ -622,7 +625,7 @@
       <c r="G4" s="10"/>
       <c r="H4" s="11"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
@@ -640,7 +643,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
@@ -658,7 +661,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>2</v>
@@ -669,7 +672,7 @@
       <c r="G7" s="10"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
@@ -687,7 +690,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
@@ -705,7 +708,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="15" t="s">
         <v>5</v>
       </c>
@@ -716,7 +719,7 @@
       <c r="G10" s="16"/>
       <c r="H10" s="17"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="9"/>
       <c r="C11" s="10" t="s">
         <v>1</v>
@@ -727,7 +730,7 @@
       <c r="G11" s="10"/>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
@@ -741,8 +744,14 @@
       <c r="H12" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J12" t="s">
+        <v>28</v>
+      </c>
+      <c r="L12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
@@ -757,7 +766,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1" t="s">
@@ -772,7 +781,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
         <v>2</v>
@@ -783,7 +792,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="11"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="9"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10" t="s">

</xml_diff>